<commit_message>
data: hourly update 2026-06-30 14:16Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-06-30.xlsx
+++ b/data/output/workbook/2026-06-30.xlsx
@@ -371,7 +371,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="9229725"/>
+    <ext cx="10125075" cy="9429750"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -401,7 +401,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="9086850"/>
+    <ext cx="10125075" cy="9467850"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -954,7 +954,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30 07:45</t>
+          <t>2026-06-30 10:15</t>
         </is>
       </c>
     </row>
@@ -7602,7 +7602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q73"/>
+  <dimension ref="A1:Q75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7619,324 +7619,170 @@
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="29" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="29" t="inlineStr">
         <is>
           <t>San Diego Padres offense vs Chicago Cubs defense</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="30" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B60" s="30" t="inlineStr">
+      <c r="B62" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C60" s="30" t="inlineStr">
+      <c r="C62" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D60" s="30" t="inlineStr">
+      <c r="D62" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E60" s="30" t="inlineStr">
+      <c r="E62" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F60" s="30" t="inlineStr">
+      <c r="F62" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G60" s="30" t="inlineStr">
+      <c r="G62" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H60" s="30" t="inlineStr">
+      <c r="H62" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I60" s="30" t="inlineStr">
+      <c r="I62" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J60" s="30" t="inlineStr">
+      <c r="J62" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K60" s="30" t="inlineStr">
+      <c r="K62" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L60" s="30" t="inlineStr">
+      <c r="L62" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M60" s="30" t="inlineStr">
+      <c r="M62" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N60" s="30" t="inlineStr">
+      <c r="N62" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O60" s="30" t="inlineStr">
+      <c r="O62" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P60" s="30" t="inlineStr">
+      <c r="P62" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q60" s="30" t="inlineStr">
+      <c r="Q62" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="31" t="inlineStr">
-        <is>
-          <t>Runs/G</t>
-        </is>
-      </c>
-      <c r="B61" s="32" t="n">
-        <v>3.987</v>
-      </c>
-      <c r="C61" s="32" t="n">
-        <v>3.733</v>
-      </c>
-      <c r="D61" s="32" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="E61" s="32" t="n">
-        <v>4.333</v>
-      </c>
-      <c r="F61" s="32" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="G61" s="32" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="H61" s="36" t="inlineStr">
-        <is>
-          <t>19th</t>
-        </is>
-      </c>
-      <c r="I61" s="32" t="inlineStr"/>
-      <c r="J61" s="33" t="inlineStr">
-        <is>
-          <t>7th</t>
-        </is>
-      </c>
-      <c r="K61" s="32" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="L61" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="M61" s="32" t="n">
-        <v>4.067</v>
-      </c>
-      <c r="N61" s="32" t="n">
-        <v>3.85</v>
-      </c>
-      <c r="O61" s="32" t="n">
-        <v>4.267</v>
-      </c>
-      <c r="P61" s="32" t="n">
-        <v>4.644</v>
-      </c>
-      <c r="Q61" s="35" t="inlineStr">
-        <is>
-          <t>Opp Runs/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="31" t="inlineStr">
-        <is>
-          <t>Hits/G</t>
-        </is>
-      </c>
-      <c r="B62" s="32" t="n">
-        <v>7.087</v>
-      </c>
-      <c r="C62" s="32" t="n">
-        <v>6.833</v>
-      </c>
-      <c r="D62" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E62" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F62" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G62" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H62" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I62" s="32" t="inlineStr"/>
-      <c r="J62" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K62" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L62" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M62" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N62" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O62" s="32" t="n">
-        <v>6.833</v>
-      </c>
-      <c r="P62" s="32" t="n">
-        <v>7.896</v>
-      </c>
-      <c r="Q62" s="35" t="inlineStr">
-        <is>
-          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Runs/G</t>
         </is>
       </c>
       <c r="B63" s="32" t="n">
-        <v>1.022</v>
+        <v>3.987</v>
       </c>
       <c r="C63" s="32" t="n">
-        <v>1.333</v>
-      </c>
-      <c r="D63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H63" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>3.733</v>
+      </c>
+      <c r="D63" s="32" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="E63" s="32" t="n">
+        <v>4.333</v>
+      </c>
+      <c r="F63" s="32" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="G63" s="32" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="H63" s="36" t="inlineStr">
+        <is>
+          <t>19th</t>
         </is>
       </c>
       <c r="I63" s="32" t="inlineStr"/>
-      <c r="J63" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J63" s="33" t="inlineStr">
+        <is>
+          <t>7th</t>
+        </is>
+      </c>
+      <c r="K63" s="32" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="L63" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="M63" s="32" t="n">
+        <v>4.067</v>
+      </c>
+      <c r="N63" s="32" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="O63" s="32" t="n">
+        <v>4.267</v>
+      </c>
+      <c r="P63" s="32" t="n">
+        <v>4.644</v>
       </c>
       <c r="Q63" s="35" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B64" s="32" t="n">
-        <v>8.348000000000001</v>
+        <v>7.087</v>
       </c>
       <c r="C64" s="32" t="n">
-        <v>9.333</v>
+        <v>6.833</v>
       </c>
       <c r="D64" s="32" t="inlineStr">
         <is>
@@ -7990,398 +7836,398 @@
         </is>
       </c>
       <c r="O64" s="32" t="n">
-        <v>7</v>
+        <v>6.833</v>
       </c>
       <c r="P64" s="32" t="n">
-        <v>7.708</v>
+        <v>7.896</v>
       </c>
       <c r="Q64" s="35" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="31" t="inlineStr">
         <is>
+          <t>HR/G</t>
+        </is>
+      </c>
+      <c r="B65" s="32" t="n">
+        <v>1.022</v>
+      </c>
+      <c r="C65" s="32" t="n">
+        <v>1.333</v>
+      </c>
+      <c r="D65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H65" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I65" s="32" t="inlineStr"/>
+      <c r="J65" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q65" s="35" t="inlineStr">
+        <is>
+          <t>Opp HR/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="31" t="inlineStr">
+        <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B66" s="32" t="n">
+        <v>8.348000000000001</v>
+      </c>
+      <c r="C66" s="32" t="n">
+        <v>9.333</v>
+      </c>
+      <c r="D66" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E66" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F66" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G66" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H66" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I66" s="32" t="inlineStr"/>
+      <c r="J66" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K66" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L66" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M66" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N66" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O66" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="P66" s="32" t="n">
+        <v>7.708</v>
+      </c>
+      <c r="Q66" s="35" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="31" t="inlineStr">
+        <is>
           <t>1st Inn R/G</t>
         </is>
       </c>
-      <c r="B65" s="32" t="n">
+      <c r="B67" s="32" t="n">
         <v>0.329</v>
       </c>
-      <c r="C65" s="32" t="n">
+      <c r="C67" s="32" t="n">
         <v>0.433</v>
       </c>
-      <c r="D65" s="32" t="n">
+      <c r="D67" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="E65" s="32" t="n">
+      <c r="E67" s="32" t="n">
         <v>0.667</v>
       </c>
-      <c r="F65" s="32" t="n">
+      <c r="F67" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="G65" s="32" t="n">
+      <c r="G67" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="H65" s="34" t="inlineStr">
+      <c r="H67" s="34" t="inlineStr">
         <is>
           <t>27th</t>
         </is>
       </c>
-      <c r="I65" s="32" t="inlineStr"/>
-      <c r="J65" s="36" t="inlineStr">
+      <c r="I67" s="32" t="inlineStr"/>
+      <c r="J67" s="36" t="inlineStr">
         <is>
           <t>14th</t>
         </is>
       </c>
-      <c r="K65" s="32" t="n">
+      <c r="K67" s="32" t="n">
         <v>0.2</v>
       </c>
-      <c r="L65" s="32" t="n">
+      <c r="L67" s="32" t="n">
         <v>0.1</v>
       </c>
-      <c r="M65" s="32" t="n">
+      <c r="M67" s="32" t="n">
         <v>0.067</v>
       </c>
-      <c r="N65" s="32" t="n">
+      <c r="N67" s="32" t="n">
         <v>0.2</v>
       </c>
-      <c r="O65" s="32" t="n">
+      <c r="O67" s="32" t="n">
         <v>0.4</v>
       </c>
-      <c r="P65" s="32" t="n">
+      <c r="P67" s="32" t="n">
         <v>0.444</v>
       </c>
-      <c r="Q65" s="35" t="inlineStr">
+      <c r="Q67" s="35" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="29" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="29" t="inlineStr">
         <is>
           <t>Chicago Cubs offense vs San Diego Padres defense</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="30" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B68" s="30" t="inlineStr">
+      <c r="B70" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C68" s="30" t="inlineStr">
+      <c r="C70" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D68" s="30" t="inlineStr">
+      <c r="D70" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E68" s="30" t="inlineStr">
+      <c r="E70" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F68" s="30" t="inlineStr">
+      <c r="F70" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G68" s="30" t="inlineStr">
+      <c r="G70" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H68" s="30" t="inlineStr">
+      <c r="H70" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I68" s="30" t="inlineStr">
+      <c r="I70" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J68" s="30" t="inlineStr">
+      <c r="J70" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K68" s="30" t="inlineStr">
+      <c r="K70" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L68" s="30" t="inlineStr">
+      <c r="L70" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M68" s="30" t="inlineStr">
+      <c r="M70" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N68" s="30" t="inlineStr">
+      <c r="N70" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O68" s="30" t="inlineStr">
+      <c r="O70" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P68" s="30" t="inlineStr">
+      <c r="P70" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q68" s="30" t="inlineStr">
+      <c r="Q70" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="31" t="inlineStr">
-        <is>
-          <t>Runs/G</t>
-        </is>
-      </c>
-      <c r="B69" s="32" t="n">
-        <v>5.027</v>
-      </c>
-      <c r="C69" s="32" t="n">
-        <v>5.367</v>
-      </c>
-      <c r="D69" s="32" t="n">
-        <v>5.7</v>
-      </c>
-      <c r="E69" s="32" t="n">
-        <v>6.267</v>
-      </c>
-      <c r="F69" s="32" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="G69" s="32" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="H69" s="36" t="inlineStr">
-        <is>
-          <t>17th</t>
-        </is>
-      </c>
-      <c r="I69" s="32" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="J69" s="34" t="inlineStr">
-        <is>
-          <t>21st</t>
-        </is>
-      </c>
-      <c r="K69" s="32" t="n">
-        <v>5</v>
-      </c>
-      <c r="L69" s="32" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="M69" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="N69" s="32" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="O69" s="32" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="P69" s="32" t="n">
-        <v>3.87</v>
-      </c>
-      <c r="Q69" s="35" t="inlineStr">
-        <is>
-          <t>Opp Runs/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="31" t="inlineStr">
-        <is>
-          <t>Hits/G</t>
-        </is>
-      </c>
-      <c r="B70" s="32" t="n">
-        <v>8.438000000000001</v>
-      </c>
-      <c r="C70" s="32" t="n">
-        <v>9.333</v>
-      </c>
-      <c r="D70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H70" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I70" s="32" t="inlineStr"/>
-      <c r="J70" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O70" s="32" t="n">
-        <v>8.333</v>
-      </c>
-      <c r="P70" s="32" t="n">
-        <v>7.848</v>
-      </c>
-      <c r="Q70" s="35" t="inlineStr">
-        <is>
-          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Runs/G</t>
         </is>
       </c>
       <c r="B71" s="32" t="n">
-        <v>1.104</v>
+        <v>5.027</v>
       </c>
       <c r="C71" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="D71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H71" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I71" s="32" t="inlineStr"/>
-      <c r="J71" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>5.367</v>
+      </c>
+      <c r="D71" s="32" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="E71" s="32" t="n">
+        <v>6.267</v>
+      </c>
+      <c r="F71" s="32" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="G71" s="32" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="H71" s="36" t="inlineStr">
+        <is>
+          <t>17th</t>
+        </is>
+      </c>
+      <c r="I71" s="32" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="J71" s="34" t="inlineStr">
+        <is>
+          <t>21st</t>
+        </is>
+      </c>
+      <c r="K71" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="L71" s="32" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="M71" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="N71" s="32" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="O71" s="32" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="P71" s="32" t="n">
+        <v>3.87</v>
       </c>
       <c r="Q71" s="35" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B72" s="32" t="n">
-        <v>8.458</v>
+        <v>8.438000000000001</v>
       </c>
       <c r="C72" s="32" t="n">
-        <v>8.833</v>
+        <v>9.333</v>
       </c>
       <c r="D72" s="32" t="inlineStr">
         <is>
@@ -8435,71 +8281,225 @@
         </is>
       </c>
       <c r="O72" s="32" t="n">
-        <v>4.833</v>
+        <v>8.333</v>
       </c>
       <c r="P72" s="32" t="n">
-        <v>8.304</v>
+        <v>7.848</v>
       </c>
       <c r="Q72" s="35" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="31" t="inlineStr">
         <is>
+          <t>HR/G</t>
+        </is>
+      </c>
+      <c r="B73" s="32" t="n">
+        <v>1.104</v>
+      </c>
+      <c r="C73" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H73" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I73" s="32" t="inlineStr"/>
+      <c r="J73" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q73" s="35" t="inlineStr">
+        <is>
+          <t>Opp HR/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="31" t="inlineStr">
+        <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B74" s="32" t="n">
+        <v>8.458</v>
+      </c>
+      <c r="C74" s="32" t="n">
+        <v>8.833</v>
+      </c>
+      <c r="D74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H74" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I74" s="32" t="inlineStr"/>
+      <c r="J74" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O74" s="32" t="n">
+        <v>4.833</v>
+      </c>
+      <c r="P74" s="32" t="n">
+        <v>8.304</v>
+      </c>
+      <c r="Q74" s="35" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="31" t="inlineStr">
+        <is>
           <t>1st Inn R/G</t>
         </is>
       </c>
-      <c r="B73" s="32" t="n">
+      <c r="B75" s="32" t="n">
         <v>0.417</v>
       </c>
-      <c r="C73" s="32" t="n">
+      <c r="C75" s="32" t="n">
         <v>0.533</v>
       </c>
-      <c r="D73" s="32" t="n">
+      <c r="D75" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="E73" s="32" t="n">
+      <c r="E75" s="32" t="n">
         <v>0.667</v>
       </c>
-      <c r="F73" s="32" t="n">
+      <c r="F75" s="32" t="n">
         <v>0.7</v>
       </c>
-      <c r="G73" s="32" t="n">
+      <c r="G75" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="H73" s="34" t="inlineStr">
+      <c r="H75" s="34" t="inlineStr">
         <is>
           <t>29th</t>
         </is>
       </c>
-      <c r="I73" s="32" t="inlineStr"/>
-      <c r="J73" s="33" t="inlineStr">
+      <c r="I75" s="32" t="inlineStr"/>
+      <c r="J75" s="33" t="inlineStr">
         <is>
           <t>6th</t>
         </is>
       </c>
-      <c r="K73" s="32" t="n">
+      <c r="K75" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="L73" s="32" t="n">
+      <c r="L75" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="M73" s="32" t="n">
+      <c r="M75" s="32" t="n">
         <v>0.533</v>
       </c>
-      <c r="N73" s="32" t="n">
+      <c r="N75" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="O73" s="32" t="n">
+      <c r="O75" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="P73" s="32" t="n">
+      <c r="P75" s="32" t="n">
         <v>0.457</v>
       </c>
-      <c r="Q73" s="35" t="inlineStr">
+      <c r="Q75" s="35" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
@@ -8848,37 +8848,37 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Kansas City Royals</t>
+          <t>Pittsburgh Pirates @ Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Under 10.5</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5517878048780488</v>
+        <v>0.4685903083700441</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-123</v>
+        <v>113</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-105</v>
+        <v>127</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -8902,7 +8902,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 55.2% (fair -123). Your call.</t>
+          <t>Model 46.9% (fair +113). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -8980,17 +8980,17 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Philadelphia Phillies</t>
+          <t>Detroit Tigers @ New York Yankees</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -9000,17 +9000,17 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.465726872246696</v>
+        <v>0.5569464454976303</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>115</v>
+        <v>-126</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>127</v>
+        <v>-111</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -9034,7 +9034,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 46.6% (fair +115). Your call.</t>
+          <t>Model 55.7% (fair -126). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -9046,7 +9046,7 @@
     <row r="10">
       <c r="A10" s="20" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B10" s="20" t="inlineStr">
@@ -9070,13 +9070,13 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.4781447963800905</v>
+        <v>0.4636563876651982</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -9100,7 +9100,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 47.8% (fair +109). Your call.</t>
+          <t>Model 46.4% (fair +116). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -9117,32 +9117,32 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Philadelphia Phillies</t>
+          <t>Tampa Bay Rays @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.5112745098039215</v>
+        <v>0.4842396313364055</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-105</v>
+        <v>107</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -9166,7 +9166,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 51.1% (fair -105). Your call.</t>
+          <t>Model 48.4% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -9178,17 +9178,17 @@
     <row r="12">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>Detroit Tigers @ New York Yankees</t>
+          <t>Texas Rangers @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="D12" s="20" t="inlineStr">
@@ -9198,17 +9198,17 @@
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.5728504504504505</v>
+        <v>0.4987980769230769</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-134</v>
+        <v>100</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>-122</v>
+        <v>108</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -9232,7 +9232,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 57.3% (fair -134). Your call.</t>
+          <t>Model 49.9% (fair +100). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -9244,37 +9244,37 @@
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Cleveland Guardians</t>
+          <t>New York Mets @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>19:07</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5245930693069306</v>
+        <v>0.5072549019607843</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-110</v>
+        <v>-103</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>-102</v>
+        <v>104</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -9298,7 +9298,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 52.5% (fair -110). Your call.</t>
+          <t>Model 50.7% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -9310,37 +9310,37 @@
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Milwaukee Brewers</t>
+          <t>San Diego Padres @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers -1.5</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4612000000000001</v>
+        <v>0.4845070422535211</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -9364,7 +9364,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 46.1% (fair +117). Your call.</t>
+          <t>Model 48.5% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -9376,17 +9376,17 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Cleveland Guardians</t>
+          <t>St. Louis Cardinals @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>17:10</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -9396,17 +9396,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>St. Louis Cardinals</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.4987980769230769</v>
+        <v>0.4318067226890757</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>100</v>
+        <v>132</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>108</v>
+        <v>138</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -9430,7 +9430,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 49.9% (fair +100). Your call.</t>
+          <t>Model 43.2% (fair +132). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -9447,12 +9447,12 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals @ Atlanta Braves</t>
+          <t>Texas Rangers @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>23:15</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
@@ -9462,17 +9462,17 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.4249590163934426</v>
+        <v>0.5335096153846154</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>135</v>
+        <v>-114</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>144</v>
+        <v>-108</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -9496,7 +9496,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 42.5% (fair +135). Your call.</t>
+          <t>Model 53.4% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -9508,7 +9508,7 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
@@ -9518,7 +9518,7 @@
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>22:35</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -9532,13 +9532,13 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4559911894273127</v>
+        <v>0.4732258064516129</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -9562,7 +9562,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 45.6% (fair +119). Your call.</t>
+          <t>Model 47.3% (fair +111). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -9574,17 +9574,17 @@
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Baltimore Orioles</t>
+          <t>New York Mets @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>23:07</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -9594,17 +9594,17 @@
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.4761290322580645</v>
+        <v>0.4935096153846154</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -9628,7 +9628,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 47.6% (fair +110). Your call.</t>
+          <t>Model 49.4% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -9640,17 +9640,17 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Cleveland Guardians</t>
+          <t>Detroit Tigers @ New York Yankees</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -9660,17 +9660,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5327307692307692</v>
+        <v>0.4195081967213115</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-114</v>
+        <v>138</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>-108</v>
+        <v>144</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -9694,7 +9694,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 53.3% (fair -114). Your call.</t>
+          <t>Model 42.0% (fair +138). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -9706,37 +9706,37 @@
     <row r="20">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>Detroit Tigers @ New York Yankees</t>
+          <t>Pittsburgh Pirates @ Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Pittsburgh Pirates +1.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4195081967213115</v>
+        <v>0.5017156862745098</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>138</v>
+        <v>-101</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>144</v>
+        <v>104</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -9760,7 +9760,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 42.0% (fair +138). Your call.</t>
+          <t>Model 50.2% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -9777,12 +9777,12 @@
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>New York Mets @ Toronto Blue Jays</t>
+          <t>Chicago White Sox @ Baltimore Orioles</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>23:07</t>
+          <t>22:35</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
@@ -9792,17 +9792,17 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4920192307692308</v>
+        <v>0.4606756756756757</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -9826,7 +9826,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 49.2% (fair +103). Your call.</t>
+          <t>Model 46.1% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -10003,13 +10003,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4559911894273127</v>
+        <v>0.4606756756756757</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -10033,7 +10033,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 45.6% (fair +119). Your call.</t>
+          <t>Model 46.1% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -10069,13 +10069,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5440299559471367</v>
+        <v>0.5393333333333333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-119</v>
+        <v>-117</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-127</v>
+        <v>-125</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -10099,7 +10099,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 54.4% (fair -119). Your call.</t>
+          <t>Model 53.9% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -10141,7 +10141,7 @@
         <v>-124</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -10207,7 +10207,7 @@
         <v>124</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -10273,7 +10273,7 @@
         <v>155</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -10339,7 +10339,7 @@
         <v>-155</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -10399,7 +10399,7 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.5327307692307692</v>
+        <v>0.5335096153846154</v>
       </c>
       <c r="G11" s="14" t="n">
         <v>-114</v>
@@ -10429,7 +10429,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 53.3% (fair -114). Your call.</t>
+          <t>Model 53.4% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -10465,13 +10465,13 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.4672946859903381</v>
+        <v>0.4664903846153846</v>
       </c>
       <c r="G12" s="14" t="n">
         <v>114</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -10495,7 +10495,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 46.7% (fair +114). Your call.</t>
+          <t>Model 46.6% (fair +114). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -10527,17 +10527,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Over 8</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5245930693069306</v>
+        <v>0.4777</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-110</v>
+        <v>109</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>-102</v>
+        <v>110</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -10561,7 +10561,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 52.5% (fair -110). Your call.</t>
+          <t>Model 47.8% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -10593,17 +10593,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Under 7.5</t>
+          <t>Under 8</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4754411764705882</v>
+        <v>0.5223</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>110</v>
+        <v>-109</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -10627,7 +10627,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 47.5% (fair +110). Your call.</t>
+          <t>Model 52.2% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -10791,17 +10791,17 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Over 9</t>
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.5112745098039215</v>
+        <v>0.4401</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-105</v>
+        <v>127</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>104</v>
+        <v>128</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -10825,7 +10825,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 51.1% (fair -105). Your call.</t>
+          <t>Model 44.0% (fair +127). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -10857,17 +10857,17 @@
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>Under 8.5</t>
+          <t>Under 9</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.48875</v>
+        <v>0.5599000000000001</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>105</v>
+        <v>-127</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>100</v>
+        <v>-104</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -10891,7 +10891,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 48.9% (fair +105). Your call.</t>
+          <t>Model 56.0% (fair -127). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -10927,13 +10927,13 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.494356862745098</v>
+        <v>0.4982514563106796</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>-104</v>
+        <v>-106</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -10957,7 +10957,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 49.4% (fair +102). Your call.</t>
+          <t>Model 49.8% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -10993,13 +10993,13 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.5056218905472637</v>
+        <v>0.5017156862745098</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>-102</v>
+        <v>-101</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -11023,7 +11023,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 50.6% (fair -102). Your call.</t>
+          <t>Model 50.2% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -11059,13 +11059,13 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4271555555555555</v>
+        <v>0.4430516431924883</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -11089,7 +11089,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 42.7% (fair +134). Your call.</t>
+          <t>Model 44.3% (fair +126). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -11125,13 +11125,13 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5728504504504505</v>
+        <v>0.5569464454976303</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-134</v>
+        <v>-126</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>-122</v>
+        <v>-111</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -11155,7 +11155,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 57.3% (fair -134). Your call.</t>
+          <t>Model 55.7% (fair -126). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -11197,7 +11197,7 @@
         <v>104</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -11263,7 +11263,7 @@
         <v>-104</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -11329,7 +11329,7 @@
         <v>120</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>167</v>
+        <v>194</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -11395,7 +11395,7 @@
         <v>-120</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>-126</v>
+        <v>176</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -11455,7 +11455,7 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.4920192307692308</v>
+        <v>0.4935096153846154</v>
       </c>
       <c r="G27" s="14" t="n">
         <v>103</v>
@@ -11485,7 +11485,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 49.2% (fair +103). Your call.</t>
+          <t>Model 49.4% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -11521,13 +11521,13 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.5080173913043478</v>
+        <v>0.506509756097561</v>
       </c>
       <c r="G28" s="14" t="n">
         <v>-103</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>-107</v>
+        <v>-105</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -11551,7 +11551,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 50.8% (fair -103). Your call.</t>
+          <t>Model 50.7% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -11583,7 +11583,7 @@
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Over 8</t>
         </is>
       </c>
       <c r="F29" s="13" t="n">
@@ -11593,7 +11593,7 @@
         <v>124</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>121</v>
+        <v>101</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -11649,7 +11649,7 @@
       </c>
       <c r="E30" s="20" t="inlineStr">
         <is>
-          <t>Under 8.5</t>
+          <t>Under 8</t>
         </is>
       </c>
       <c r="F30" s="13" t="n">
@@ -11791,7 +11791,7 @@
         <v>-188</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="I32" s="13">
         <f>IF($H$32="","",IF($H$32&lt;0,-$H$32/(-$H$32+100),100/($H$32+100)))</f>
@@ -11857,7 +11857,7 @@
         <v>-113</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="I33" s="13">
         <f>IF($H$33="","",IF($H$33&lt;0,-$H$33/(-$H$33+100),100/($H$33+100)))</f>
@@ -11923,7 +11923,7 @@
         <v>113</v>
       </c>
       <c r="H34" s="15" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="I34" s="13">
         <f>IF($H$34="","",IF($H$34&lt;0,-$H$34/(-$H$34+100),100/($H$34+100)))</f>
@@ -11989,7 +11989,7 @@
         <v>116</v>
       </c>
       <c r="H35" s="15" t="n">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="I35" s="13">
         <f>IF($H$35="","",IF($H$35&lt;0,-$H$35/(-$H$35+100),100/($H$35+100)))</f>
@@ -12055,7 +12055,7 @@
         <v>-116</v>
       </c>
       <c r="H36" s="15" t="n">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="I36" s="13">
         <f>IF($H$36="","",IF($H$36&lt;0,-$H$36/(-$H$36+100),100/($H$36+100)))</f>
@@ -12121,7 +12121,7 @@
         <v>191</v>
       </c>
       <c r="H37" s="15" t="n">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="I37" s="13">
         <f>IF($H$37="","",IF($H$37&lt;0,-$H$37/(-$H$37+100),100/($H$37+100)))</f>
@@ -12187,7 +12187,7 @@
         <v>-191</v>
       </c>
       <c r="H38" s="15" t="n">
-        <v>-115</v>
+        <v>-121</v>
       </c>
       <c r="I38" s="13">
         <f>IF($H$38="","",IF($H$38&lt;0,-$H$38/(-$H$38+100),100/($H$38+100)))</f>
@@ -12247,13 +12247,13 @@
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>0.4249590163934426</v>
+        <v>0.4318067226890757</v>
       </c>
       <c r="G39" s="14" t="n">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="H39" s="15" t="n">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="I39" s="13">
         <f>IF($H$39="","",IF($H$39&lt;0,-$H$39/(-$H$39+100),100/($H$39+100)))</f>
@@ -12277,7 +12277,7 @@
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>Model 42.5% (fair +135). Your call.</t>
+          <t>Model 43.2% (fair +132). Your call.</t>
         </is>
       </c>
       <c r="O39" s="15" t="n"/>
@@ -12313,13 +12313,13 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.5749991701244813</v>
+        <v>0.5682063829787234</v>
       </c>
       <c r="G40" s="14" t="n">
+        <v>-132</v>
+      </c>
+      <c r="H40" s="15" t="n">
         <v>-135</v>
-      </c>
-      <c r="H40" s="15" t="n">
-        <v>-141</v>
       </c>
       <c r="I40" s="13">
         <f>IF($H$40="","",IF($H$40&lt;0,-$H$40/(-$H$40+100),100/($H$40+100)))</f>
@@ -12343,7 +12343,7 @@
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>Model 57.5% (fair -135). Your call.</t>
+          <t>Model 56.8% (fair -132). Your call.</t>
         </is>
       </c>
       <c r="O40" s="15" t="n"/>
@@ -12375,17 +12375,17 @@
       </c>
       <c r="E41" s="12" t="inlineStr">
         <is>
-          <t>Over 10</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>0.3333</v>
+        <v>0.4017</v>
       </c>
       <c r="G41" s="14" t="n">
-        <v>200</v>
+        <v>149</v>
       </c>
       <c r="H41" s="15" t="n">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="I41" s="13">
         <f>IF($H$41="","",IF($H$41&lt;0,-$H$41/(-$H$41+100),100/($H$41+100)))</f>
@@ -12409,7 +12409,7 @@
       </c>
       <c r="N41" s="19" t="inlineStr">
         <is>
-          <t>Model 33.3% (fair +200). Your call.</t>
+          <t>Model 40.2% (fair +149). Your call.</t>
         </is>
       </c>
       <c r="O41" s="15" t="n"/>
@@ -12441,17 +12441,17 @@
       </c>
       <c r="E42" s="20" t="inlineStr">
         <is>
-          <t>Under 10</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.6667000000000001</v>
+        <v>0.5983000000000001</v>
       </c>
       <c r="G42" s="14" t="n">
-        <v>-200</v>
+        <v>-149</v>
       </c>
       <c r="H42" s="15" t="n">
-        <v>-104</v>
+        <v>107</v>
       </c>
       <c r="I42" s="13">
         <f>IF($H$42="","",IF($H$42&lt;0,-$H$42/(-$H$42+100),100/($H$42+100)))</f>
@@ -12475,7 +12475,7 @@
       </c>
       <c r="N42" s="19" t="inlineStr">
         <is>
-          <t>Model 66.7% (fair -200). Your call.</t>
+          <t>Model 59.8% (fair -149). Your call.</t>
         </is>
       </c>
       <c r="O42" s="15" t="n"/>
@@ -12517,7 +12517,7 @@
         <v>142</v>
       </c>
       <c r="H43" s="15" t="n">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="I43" s="13">
         <f>IF($H$43="","",IF($H$43&lt;0,-$H$43/(-$H$43+100),100/($H$43+100)))</f>
@@ -12583,7 +12583,7 @@
         <v>-142</v>
       </c>
       <c r="H44" s="15" t="n">
-        <v>104</v>
+        <v>-105</v>
       </c>
       <c r="I44" s="13">
         <f>IF($H$44="","",IF($H$44&lt;0,-$H$44/(-$H$44+100),100/($H$44+100)))</f>
@@ -12643,13 +12643,13 @@
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>0.5218909090909091</v>
+        <v>0.5157883720930233</v>
       </c>
       <c r="G45" s="14" t="n">
-        <v>-109</v>
+        <v>-107</v>
       </c>
       <c r="H45" s="15" t="n">
-        <v>-120</v>
+        <v>-115</v>
       </c>
       <c r="I45" s="13">
         <f>IF($H$45="","",IF($H$45&lt;0,-$H$45/(-$H$45+100),100/($H$45+100)))</f>
@@ -12673,7 +12673,7 @@
       </c>
       <c r="N45" s="19" t="inlineStr">
         <is>
-          <t>Model 52.2% (fair -109). Your call.</t>
+          <t>Model 51.6% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O45" s="15" t="n"/>
@@ -12709,13 +12709,13 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.4781447963800905</v>
+        <v>0.4842396313364055</v>
       </c>
       <c r="G46" s="14" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H46" s="15" t="n">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="I46" s="13">
         <f>IF($H$46="","",IF($H$46&lt;0,-$H$46/(-$H$46+100),100/($H$46+100)))</f>
@@ -12739,7 +12739,7 @@
       </c>
       <c r="N46" s="19" t="inlineStr">
         <is>
-          <t>Model 47.8% (fair +109). Your call.</t>
+          <t>Model 48.4% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O46" s="15" t="n"/>
@@ -12775,13 +12775,13 @@
         </is>
       </c>
       <c r="F47" s="13" t="n">
-        <v>0.4482159624413146</v>
+        <v>0.3925</v>
       </c>
       <c r="G47" s="14" t="n">
-        <v>123</v>
+        <v>155</v>
       </c>
       <c r="H47" s="15" t="n">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="I47" s="13">
         <f>IF($H$47="","",IF($H$47&lt;0,-$H$47/(-$H$47+100),100/($H$47+100)))</f>
@@ -12805,7 +12805,7 @@
       </c>
       <c r="N47" s="19" t="inlineStr">
         <is>
-          <t>Model 44.8% (fair +123). Your call.</t>
+          <t>Model 39.2% (fair +155). Your call.</t>
         </is>
       </c>
       <c r="O47" s="15" t="n"/>
@@ -12841,13 +12841,13 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.5517878048780488</v>
+        <v>0.6074999999999999</v>
       </c>
       <c r="G48" s="14" t="n">
-        <v>-123</v>
+        <v>-155</v>
       </c>
       <c r="H48" s="15" t="n">
-        <v>-105</v>
+        <v>108</v>
       </c>
       <c r="I48" s="13">
         <f>IF($H$48="","",IF($H$48&lt;0,-$H$48/(-$H$48+100),100/($H$48+100)))</f>
@@ -12871,7 +12871,7 @@
       </c>
       <c r="N48" s="19" t="inlineStr">
         <is>
-          <t>Model 55.2% (fair -123). Your call.</t>
+          <t>Model 60.7% (fair -155). Your call.</t>
         </is>
       </c>
       <c r="O48" s="15" t="n"/>
@@ -12907,10 +12907,10 @@
         </is>
       </c>
       <c r="F49" s="13" t="n">
-        <v>0.381015625</v>
+        <v>0.3828515625</v>
       </c>
       <c r="G49" s="14" t="n">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H49" s="15" t="n">
         <v>156</v>
@@ -12937,7 +12937,7 @@
       </c>
       <c r="N49" s="19" t="inlineStr">
         <is>
-          <t>Model 38.1% (fair +162). Your call.</t>
+          <t>Model 38.3% (fair +161). Your call.</t>
         </is>
       </c>
       <c r="O49" s="15" t="n"/>
@@ -12973,13 +12973,13 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.6189661596958175</v>
+        <v>0.6171798449612403</v>
       </c>
       <c r="G50" s="14" t="n">
-        <v>-162</v>
+        <v>-161</v>
       </c>
       <c r="H50" s="15" t="n">
-        <v>-163</v>
+        <v>-158</v>
       </c>
       <c r="I50" s="13">
         <f>IF($H$50="","",IF($H$50&lt;0,-$H$50/(-$H$50+100),100/($H$50+100)))</f>
@@ -13003,7 +13003,7 @@
       </c>
       <c r="N50" s="19" t="inlineStr">
         <is>
-          <t>Model 61.9% (fair -162). Your call.</t>
+          <t>Model 61.7% (fair -161). Your call.</t>
         </is>
       </c>
       <c r="O50" s="15" t="n"/>
@@ -13035,7 +13035,7 @@
       </c>
       <c r="E51" s="12" t="inlineStr">
         <is>
-          <t>Over 9</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F51" s="13" t="n">
@@ -13045,7 +13045,7 @@
         <v>115</v>
       </c>
       <c r="H51" s="15" t="n">
-        <v>107</v>
+        <v>127</v>
       </c>
       <c r="I51" s="13">
         <f>IF($H$51="","",IF($H$51&lt;0,-$H$51/(-$H$51+100),100/($H$51+100)))</f>
@@ -13101,7 +13101,7 @@
       </c>
       <c r="E52" s="20" t="inlineStr">
         <is>
-          <t>Under 9</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F52" s="13" t="n">
@@ -13111,7 +13111,7 @@
         <v>-115</v>
       </c>
       <c r="H52" s="15" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="I52" s="13">
         <f>IF($H$52="","",IF($H$52&lt;0,-$H$52/(-$H$52+100),100/($H$52+100)))</f>
@@ -13171,13 +13171,13 @@
         </is>
       </c>
       <c r="F53" s="13" t="n">
-        <v>0.4612000000000001</v>
+        <v>0.4955</v>
       </c>
       <c r="G53" s="14" t="n">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="H53" s="15" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="I53" s="13">
         <f>IF($H$53="","",IF($H$53&lt;0,-$H$53/(-$H$53+100),100/($H$53+100)))</f>
@@ -13201,7 +13201,7 @@
       </c>
       <c r="N53" s="19" t="inlineStr">
         <is>
-          <t>Model 46.1% (fair +117). Your call.</t>
+          <t>Model 49.5% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O53" s="15" t="n"/>
@@ -13237,13 +13237,13 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.538826872246696</v>
+        <v>0.5044999999999999</v>
       </c>
       <c r="G54" s="14" t="n">
-        <v>-117</v>
+        <v>-102</v>
       </c>
       <c r="H54" s="15" t="n">
-        <v>-127</v>
+        <v>110</v>
       </c>
       <c r="I54" s="13">
         <f>IF($H$54="","",IF($H$54&lt;0,-$H$54/(-$H$54+100),100/($H$54+100)))</f>
@@ -13267,7 +13267,7 @@
       </c>
       <c r="N54" s="19" t="inlineStr">
         <is>
-          <t>Model 53.9% (fair -117). Your call.</t>
+          <t>Model 50.4% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O54" s="15" t="n"/>
@@ -13303,10 +13303,10 @@
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>0.4234873949579832</v>
+        <v>0.4221008403361344</v>
       </c>
       <c r="G55" s="14" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H55" s="15" t="n">
         <v>138</v>
@@ -13333,7 +13333,7 @@
       </c>
       <c r="N55" s="19" t="inlineStr">
         <is>
-          <t>Model 42.3% (fair +136). Your call.</t>
+          <t>Model 42.2% (fair +137). Your call.</t>
         </is>
       </c>
       <c r="O55" s="15" t="n"/>
@@ -13369,13 +13369,13 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.5764689075630252</v>
+        <v>0.5779244813278008</v>
       </c>
       <c r="G56" s="14" t="n">
-        <v>-136</v>
+        <v>-137</v>
       </c>
       <c r="H56" s="15" t="n">
-        <v>-138</v>
+        <v>-141</v>
       </c>
       <c r="I56" s="13">
         <f>IF($H$56="","",IF($H$56&lt;0,-$H$56/(-$H$56+100),100/($H$56+100)))</f>
@@ -13399,7 +13399,7 @@
       </c>
       <c r="N56" s="19" t="inlineStr">
         <is>
-          <t>Model 57.6% (fair -136). Your call.</t>
+          <t>Model 57.8% (fair -137). Your call.</t>
         </is>
       </c>
       <c r="O56" s="15" t="n"/>
@@ -13441,7 +13441,7 @@
         <v>336</v>
       </c>
       <c r="H57" s="15" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="I57" s="13">
         <f>IF($H$57="","",IF($H$57&lt;0,-$H$57/(-$H$57+100),100/($H$57+100)))</f>
@@ -13507,7 +13507,7 @@
         <v>-336</v>
       </c>
       <c r="H58" s="15" t="n">
-        <v>-101</v>
+        <v>106</v>
       </c>
       <c r="I58" s="13">
         <f>IF($H$58="","",IF($H$58&lt;0,-$H$58/(-$H$58+100),100/($H$58+100)))</f>
@@ -13567,13 +13567,13 @@
         </is>
       </c>
       <c r="F59" s="13" t="n">
-        <v>0.4289270386266094</v>
+        <v>0.4285</v>
       </c>
       <c r="G59" s="14" t="n">
         <v>133</v>
       </c>
       <c r="H59" s="15" t="n">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="I59" s="13">
         <f>IF($H$59="","",IF($H$59&lt;0,-$H$59/(-$H$59+100),100/($H$59+100)))</f>
@@ -13633,13 +13633,13 @@
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.5710437768240343</v>
+        <v>0.5715</v>
       </c>
       <c r="G60" s="14" t="n">
         <v>-133</v>
       </c>
       <c r="H60" s="15" t="n">
-        <v>-133</v>
+        <v>-101</v>
       </c>
       <c r="I60" s="13">
         <f>IF($H$60="","",IF($H$60&lt;0,-$H$60/(-$H$60+100),100/($H$60+100)))</f>
@@ -14339,10 +14339,10 @@
         </is>
       </c>
       <c r="F71" s="13" t="n">
-        <v>0.4761290322580645</v>
+        <v>0.4732258064516129</v>
       </c>
       <c r="G71" s="14" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H71" s="15" t="n">
         <v>117</v>
@@ -14369,7 +14369,7 @@
       </c>
       <c r="N71" s="19" t="inlineStr">
         <is>
-          <t>Model 47.6% (fair +110). Your call.</t>
+          <t>Model 47.3% (fair +111). Your call.</t>
         </is>
       </c>
       <c r="O71" s="15" t="n"/>
@@ -14405,13 +14405,13 @@
         </is>
       </c>
       <c r="F72" s="13" t="n">
-        <v>0.5238855855855856</v>
+        <v>0.5267422907488987</v>
       </c>
       <c r="G72" s="14" t="n">
-        <v>-110</v>
+        <v>-111</v>
       </c>
       <c r="H72" s="15" t="n">
-        <v>-122</v>
+        <v>-127</v>
       </c>
       <c r="I72" s="13">
         <f>IF($H$72="","",IF($H$72&lt;0,-$H$72/(-$H$72+100),100/($H$72+100)))</f>
@@ -14435,7 +14435,7 @@
       </c>
       <c r="N72" s="19" t="inlineStr">
         <is>
-          <t>Model 52.4% (fair -110). Your call.</t>
+          <t>Model 52.7% (fair -111). Your call.</t>
         </is>
       </c>
       <c r="O72" s="15" t="n"/>
@@ -14609,7 +14609,7 @@
         <v>109</v>
       </c>
       <c r="H75" s="15" t="n">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="I75" s="13">
         <f>IF($H$75="","",IF($H$75&lt;0,-$H$75/(-$H$75+100),100/($H$75+100)))</f>
@@ -14867,13 +14867,13 @@
         </is>
       </c>
       <c r="F79" s="13" t="n">
-        <v>0.4883173076923077</v>
+        <v>0.4845070422535211</v>
       </c>
       <c r="G79" s="14" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H79" s="15" t="n">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I79" s="13">
         <f>IF($H$79="","",IF($H$79&lt;0,-$H$79/(-$H$79+100),100/($H$79+100)))</f>
@@ -14897,7 +14897,7 @@
       </c>
       <c r="N79" s="19" t="inlineStr">
         <is>
-          <t>Model 48.8% (fair +105). Your call.</t>
+          <t>Model 48.5% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O79" s="15" t="n"/>
@@ -14933,10 +14933,10 @@
         </is>
       </c>
       <c r="F80" s="13" t="n">
-        <v>0.51165</v>
+        <v>0.5154923076923077</v>
       </c>
       <c r="G80" s="14" t="n">
-        <v>-105</v>
+        <v>-106</v>
       </c>
       <c r="H80" s="15" t="n">
         <v>-108</v>
@@ -14963,7 +14963,7 @@
       </c>
       <c r="N80" s="19" t="inlineStr">
         <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
+          <t>Model 51.5% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O80" s="15" t="n"/>
@@ -14999,10 +14999,10 @@
         </is>
       </c>
       <c r="F81" s="13" t="n">
-        <v>0.5208</v>
+        <v>0.5072549019607843</v>
       </c>
       <c r="G81" s="14" t="n">
-        <v>-109</v>
+        <v>-103</v>
       </c>
       <c r="H81" s="15" t="n">
         <v>104</v>
@@ -15029,7 +15029,7 @@
       </c>
       <c r="N81" s="19" t="inlineStr">
         <is>
-          <t>Model 52.1% (fair -109). Your call.</t>
+          <t>Model 50.7% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O81" s="15" t="n"/>
@@ -15065,13 +15065,13 @@
         </is>
       </c>
       <c r="F82" s="13" t="n">
-        <v>0.4793</v>
+        <v>0.4927450980392157</v>
       </c>
       <c r="G82" s="14" t="n">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="H82" s="15" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I82" s="13">
         <f>IF($H$82="","",IF($H$82&lt;0,-$H$82/(-$H$82+100),100/($H$82+100)))</f>
@@ -15095,7 +15095,7 @@
       </c>
       <c r="N82" s="19" t="inlineStr">
         <is>
-          <t>Model 47.9% (fair +109). Your call.</t>
+          <t>Model 49.3% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O82" s="15" t="n"/>
@@ -15131,10 +15131,10 @@
         </is>
       </c>
       <c r="F83" s="13" t="n">
-        <v>0.465726872246696</v>
+        <v>0.4685903083700441</v>
       </c>
       <c r="G83" s="14" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H83" s="15" t="n">
         <v>127</v>
@@ -15161,7 +15161,7 @@
       </c>
       <c r="N83" s="19" t="inlineStr">
         <is>
-          <t>Model 46.6% (fair +115). Your call.</t>
+          <t>Model 46.9% (fair +113). Your call.</t>
         </is>
       </c>
       <c r="O83" s="15" t="n"/>
@@ -15197,13 +15197,13 @@
         </is>
       </c>
       <c r="F84" s="13" t="n">
-        <v>0.534295154185022</v>
+        <v>0.5314144144144144</v>
       </c>
       <c r="G84" s="14" t="n">
-        <v>-115</v>
+        <v>-113</v>
       </c>
       <c r="H84" s="15" t="n">
-        <v>-127</v>
+        <v>-122</v>
       </c>
       <c r="I84" s="13">
         <f>IF($H$84="","",IF($H$84&lt;0,-$H$84/(-$H$84+100),100/($H$84+100)))</f>
@@ -15227,7 +15227,7 @@
       </c>
       <c r="N84" s="19" t="inlineStr">
         <is>
-          <t>Model 53.4% (fair -115). Your call.</t>
+          <t>Model 53.1% (fair -113). Your call.</t>
         </is>
       </c>
       <c r="O84" s="15" t="n"/>
@@ -15395,10 +15395,10 @@
         </is>
       </c>
       <c r="F87" s="13" t="n">
-        <v>0.5016</v>
+        <v>0.5363603603603604</v>
       </c>
       <c r="G87" s="14" t="n">
-        <v>-101</v>
+        <v>-116</v>
       </c>
       <c r="H87" s="15" t="n">
         <v>-122</v>
@@ -15425,7 +15425,7 @@
       </c>
       <c r="N87" s="19" t="inlineStr">
         <is>
-          <t>Model 50.2% (fair -101). Your call.</t>
+          <t>Model 53.6% (fair -116). Your call.</t>
         </is>
       </c>
       <c r="O87" s="15" t="n"/>
@@ -15461,13 +15461,13 @@
         </is>
       </c>
       <c r="F88" s="13" t="n">
-        <v>0.4984</v>
+        <v>0.4636563876651982</v>
       </c>
       <c r="G88" s="14" t="n">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="H88" s="15" t="n">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="I88" s="13">
         <f>IF($H$88="","",IF($H$88&lt;0,-$H$88/(-$H$88+100),100/($H$88+100)))</f>
@@ -15491,7 +15491,7 @@
       </c>
       <c r="N88" s="19" t="inlineStr">
         <is>
-          <t>Model 49.8% (fair +101). Your call.</t>
+          <t>Model 46.4% (fair +116). Your call.</t>
         </is>
       </c>
       <c r="O88" s="15" t="n"/>
@@ -17897,7 +17897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q73"/>
+  <dimension ref="A1:Q75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17914,328 +17914,174 @@
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="29" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="29" t="inlineStr">
         <is>
           <t>Texas Rangers offense vs Cleveland Guardians defense</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="30" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B60" s="30" t="inlineStr">
+      <c r="B62" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C60" s="30" t="inlineStr">
+      <c r="C62" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D60" s="30" t="inlineStr">
+      <c r="D62" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E60" s="30" t="inlineStr">
+      <c r="E62" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F60" s="30" t="inlineStr">
+      <c r="F62" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G60" s="30" t="inlineStr">
+      <c r="G62" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H60" s="30" t="inlineStr">
+      <c r="H62" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I60" s="30" t="inlineStr">
+      <c r="I62" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J60" s="30" t="inlineStr">
+      <c r="J62" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K60" s="30" t="inlineStr">
+      <c r="K62" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L60" s="30" t="inlineStr">
+      <c r="L62" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M60" s="30" t="inlineStr">
+      <c r="M62" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N60" s="30" t="inlineStr">
+      <c r="N62" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O60" s="30" t="inlineStr">
+      <c r="O62" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P60" s="30" t="inlineStr">
+      <c r="P62" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q60" s="30" t="inlineStr">
+      <c r="Q62" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="31" t="inlineStr">
-        <is>
-          <t>Runs/G</t>
-        </is>
-      </c>
-      <c r="B61" s="32" t="n">
-        <v>4.15</v>
-      </c>
-      <c r="C61" s="32" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="D61" s="32" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="E61" s="32" t="n">
-        <v>4.467</v>
-      </c>
-      <c r="F61" s="32" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="G61" s="32" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="H61" s="33" t="inlineStr">
-        <is>
-          <t>8th</t>
-        </is>
-      </c>
-      <c r="I61" s="32" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="J61" s="36" t="inlineStr">
-        <is>
-          <t>12th</t>
-        </is>
-      </c>
-      <c r="K61" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="L61" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="M61" s="32" t="n">
-        <v>3.733</v>
-      </c>
-      <c r="N61" s="32" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="O61" s="32" t="n">
-        <v>4.533</v>
-      </c>
-      <c r="P61" s="32" t="n">
-        <v>4.133</v>
-      </c>
-      <c r="Q61" s="35" t="inlineStr">
-        <is>
-          <t>Opp Runs/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="31" t="inlineStr">
-        <is>
-          <t>Hits/G</t>
-        </is>
-      </c>
-      <c r="B62" s="32" t="n">
-        <v>7.816</v>
-      </c>
-      <c r="C62" s="32" t="n">
-        <v>9.167</v>
-      </c>
-      <c r="D62" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E62" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F62" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G62" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H62" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I62" s="32" t="inlineStr"/>
-      <c r="J62" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K62" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L62" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M62" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N62" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O62" s="32" t="n">
-        <v>10.429</v>
-      </c>
-      <c r="P62" s="32" t="n">
-        <v>7.939</v>
-      </c>
-      <c r="Q62" s="35" t="inlineStr">
-        <is>
-          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Runs/G</t>
         </is>
       </c>
       <c r="B63" s="32" t="n">
-        <v>1.041</v>
+        <v>4.15</v>
       </c>
       <c r="C63" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="D63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H63" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I63" s="32" t="inlineStr"/>
-      <c r="J63" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P63" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>4.4</v>
+      </c>
+      <c r="D63" s="32" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E63" s="32" t="n">
+        <v>4.467</v>
+      </c>
+      <c r="F63" s="32" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G63" s="32" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="H63" s="33" t="inlineStr">
+        <is>
+          <t>8th</t>
+        </is>
+      </c>
+      <c r="I63" s="32" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="J63" s="36" t="inlineStr">
+        <is>
+          <t>12th</t>
+        </is>
+      </c>
+      <c r="K63" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="L63" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="M63" s="32" t="n">
+        <v>3.733</v>
+      </c>
+      <c r="N63" s="32" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="O63" s="32" t="n">
+        <v>4.533</v>
+      </c>
+      <c r="P63" s="32" t="n">
+        <v>4.133</v>
       </c>
       <c r="Q63" s="35" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B64" s="32" t="n">
-        <v>8.592000000000001</v>
+        <v>7.816</v>
       </c>
       <c r="C64" s="32" t="n">
-        <v>8.833</v>
+        <v>9.167</v>
       </c>
       <c r="D64" s="32" t="inlineStr">
         <is>
@@ -18289,398 +18135,398 @@
         </is>
       </c>
       <c r="O64" s="32" t="n">
-        <v>9</v>
+        <v>10.429</v>
       </c>
       <c r="P64" s="32" t="n">
-        <v>9.388</v>
+        <v>7.939</v>
       </c>
       <c r="Q64" s="35" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="31" t="inlineStr">
         <is>
+          <t>HR/G</t>
+        </is>
+      </c>
+      <c r="B65" s="32" t="n">
+        <v>1.041</v>
+      </c>
+      <c r="C65" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H65" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I65" s="32" t="inlineStr"/>
+      <c r="J65" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q65" s="35" t="inlineStr">
+        <is>
+          <t>Opp HR/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="31" t="inlineStr">
+        <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B66" s="32" t="n">
+        <v>8.592000000000001</v>
+      </c>
+      <c r="C66" s="32" t="n">
+        <v>8.833</v>
+      </c>
+      <c r="D66" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E66" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F66" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G66" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H66" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I66" s="32" t="inlineStr"/>
+      <c r="J66" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K66" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L66" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M66" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N66" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O66" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="P66" s="32" t="n">
+        <v>9.388</v>
+      </c>
+      <c r="Q66" s="35" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="31" t="inlineStr">
+        <is>
           <t>1st Inn R/G</t>
         </is>
       </c>
-      <c r="B65" s="32" t="n">
+      <c r="B67" s="32" t="n">
         <v>0.63</v>
       </c>
-      <c r="C65" s="32" t="n">
+      <c r="C67" s="32" t="n">
         <v>0.867</v>
       </c>
-      <c r="D65" s="32" t="n">
+      <c r="D67" s="32" t="n">
         <v>0.75</v>
       </c>
-      <c r="E65" s="32" t="n">
+      <c r="E67" s="32" t="n">
         <v>0.867</v>
       </c>
-      <c r="F65" s="32" t="n">
+      <c r="F67" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="G65" s="32" t="n">
+      <c r="G67" s="32" t="n">
         <v>1.2</v>
       </c>
-      <c r="H65" s="33" t="inlineStr">
+      <c r="H67" s="33" t="inlineStr">
         <is>
           <t>3rd</t>
         </is>
       </c>
-      <c r="I65" s="32" t="inlineStr">
+      <c r="I67" s="32" t="inlineStr">
         <is>
           <t>★</t>
         </is>
       </c>
-      <c r="J65" s="33" t="inlineStr">
+      <c r="J67" s="33" t="inlineStr">
         <is>
           <t>8th</t>
         </is>
       </c>
-      <c r="K65" s="32" t="n">
+      <c r="K67" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="L65" s="32" t="n">
+      <c r="L67" s="32" t="n">
         <v>0.2</v>
       </c>
-      <c r="M65" s="32" t="n">
+      <c r="M67" s="32" t="n">
         <v>0.4</v>
       </c>
-      <c r="N65" s="32" t="n">
+      <c r="N67" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="O65" s="32" t="n">
+      <c r="O67" s="32" t="n">
         <v>0.467</v>
       </c>
-      <c r="P65" s="32" t="n">
+      <c r="P67" s="32" t="n">
         <v>0.375</v>
       </c>
-      <c r="Q65" s="35" t="inlineStr">
+      <c r="Q67" s="35" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="29" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="29" t="inlineStr">
         <is>
           <t>Cleveland Guardians offense vs Texas Rangers defense</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="30" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B68" s="30" t="inlineStr">
+      <c r="B70" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C68" s="30" t="inlineStr">
+      <c r="C70" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D68" s="30" t="inlineStr">
+      <c r="D70" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E68" s="30" t="inlineStr">
+      <c r="E70" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F68" s="30" t="inlineStr">
+      <c r="F70" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G68" s="30" t="inlineStr">
+      <c r="G70" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H68" s="30" t="inlineStr">
+      <c r="H70" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I68" s="30" t="inlineStr">
+      <c r="I70" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J68" s="30" t="inlineStr">
+      <c r="J70" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K68" s="30" t="inlineStr">
+      <c r="K70" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L68" s="30" t="inlineStr">
+      <c r="L70" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M68" s="30" t="inlineStr">
+      <c r="M70" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N68" s="30" t="inlineStr">
+      <c r="N70" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O68" s="30" t="inlineStr">
+      <c r="O70" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P68" s="30" t="inlineStr">
+      <c r="P70" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q68" s="30" t="inlineStr">
+      <c r="Q70" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="31" t="inlineStr">
-        <is>
-          <t>Runs/G</t>
-        </is>
-      </c>
-      <c r="B69" s="32" t="n">
-        <v>3.88</v>
-      </c>
-      <c r="C69" s="32" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="D69" s="32" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="E69" s="32" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="F69" s="32" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="G69" s="32" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="H69" s="34" t="inlineStr">
-        <is>
-          <t>22nd</t>
-        </is>
-      </c>
-      <c r="I69" s="32" t="inlineStr"/>
-      <c r="J69" s="33" t="inlineStr">
-        <is>
-          <t>8th</t>
-        </is>
-      </c>
-      <c r="K69" s="32" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="L69" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="M69" s="32" t="n">
-        <v>5.067</v>
-      </c>
-      <c r="N69" s="32" t="n">
-        <v>5.15</v>
-      </c>
-      <c r="O69" s="32" t="n">
-        <v>4.533</v>
-      </c>
-      <c r="P69" s="32" t="n">
-        <v>4.138</v>
-      </c>
-      <c r="Q69" s="35" t="inlineStr">
-        <is>
-          <t>Opp Runs/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="31" t="inlineStr">
-        <is>
-          <t>Hits/G</t>
-        </is>
-      </c>
-      <c r="B70" s="32" t="n">
-        <v>7.735</v>
-      </c>
-      <c r="C70" s="32" t="n">
-        <v>9.143000000000001</v>
-      </c>
-      <c r="D70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H70" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I70" s="32" t="inlineStr"/>
-      <c r="J70" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O70" s="32" t="n">
-        <v>8.167</v>
-      </c>
-      <c r="P70" s="32" t="n">
-        <v>7.673</v>
-      </c>
-      <c r="Q70" s="35" t="inlineStr">
-        <is>
-          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Runs/G</t>
         </is>
       </c>
       <c r="B71" s="32" t="n">
-        <v>0.959</v>
+        <v>3.88</v>
       </c>
       <c r="C71" s="32" t="n">
-        <v>0.286</v>
-      </c>
-      <c r="D71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H71" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>3.4</v>
+      </c>
+      <c r="D71" s="32" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="E71" s="32" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F71" s="32" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G71" s="32" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="H71" s="34" t="inlineStr">
+        <is>
+          <t>22nd</t>
         </is>
       </c>
       <c r="I71" s="32" t="inlineStr"/>
-      <c r="J71" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J71" s="33" t="inlineStr">
+        <is>
+          <t>8th</t>
+        </is>
+      </c>
+      <c r="K71" s="32" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="L71" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="M71" s="32" t="n">
+        <v>5.067</v>
+      </c>
+      <c r="N71" s="32" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="O71" s="32" t="n">
+        <v>4.533</v>
+      </c>
+      <c r="P71" s="32" t="n">
+        <v>4.138</v>
       </c>
       <c r="Q71" s="35" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B72" s="32" t="n">
-        <v>8</v>
+        <v>7.735</v>
       </c>
       <c r="C72" s="32" t="n">
-        <v>9.429</v>
+        <v>9.143000000000001</v>
       </c>
       <c r="D72" s="32" t="inlineStr">
         <is>
@@ -18734,71 +18580,225 @@
         </is>
       </c>
       <c r="O72" s="32" t="n">
-        <v>9.167</v>
+        <v>8.167</v>
       </c>
       <c r="P72" s="32" t="n">
-        <v>8.571</v>
+        <v>7.673</v>
       </c>
       <c r="Q72" s="35" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="31" t="inlineStr">
         <is>
+          <t>HR/G</t>
+        </is>
+      </c>
+      <c r="B73" s="32" t="n">
+        <v>0.959</v>
+      </c>
+      <c r="C73" s="32" t="n">
+        <v>0.286</v>
+      </c>
+      <c r="D73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H73" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I73" s="32" t="inlineStr"/>
+      <c r="J73" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q73" s="35" t="inlineStr">
+        <is>
+          <t>Opp HR/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="31" t="inlineStr">
+        <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B74" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C74" s="32" t="n">
+        <v>9.429</v>
+      </c>
+      <c r="D74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H74" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I74" s="32" t="inlineStr"/>
+      <c r="J74" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O74" s="32" t="n">
+        <v>9.167</v>
+      </c>
+      <c r="P74" s="32" t="n">
+        <v>8.571</v>
+      </c>
+      <c r="Q74" s="35" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="31" t="inlineStr">
+        <is>
           <t>1st Inn R/G</t>
         </is>
       </c>
-      <c r="B73" s="32" t="n">
+      <c r="B75" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="C73" s="32" t="n">
+      <c r="C75" s="32" t="n">
         <v>0.3</v>
       </c>
-      <c r="D73" s="32" t="n">
+      <c r="D75" s="32" t="n">
         <v>0.15</v>
       </c>
-      <c r="E73" s="32" t="n">
+      <c r="E75" s="32" t="n">
         <v>0.133</v>
       </c>
-      <c r="F73" s="32" t="n">
+      <c r="F75" s="32" t="n">
         <v>0.2</v>
       </c>
-      <c r="G73" s="32" t="n">
+      <c r="G75" s="32" t="n">
         <v>0.2</v>
       </c>
-      <c r="H73" s="36" t="inlineStr">
+      <c r="H75" s="36" t="inlineStr">
         <is>
           <t>19th</t>
         </is>
       </c>
-      <c r="I73" s="32" t="inlineStr"/>
-      <c r="J73" s="33" t="inlineStr">
+      <c r="I75" s="32" t="inlineStr"/>
+      <c r="J75" s="33" t="inlineStr">
         <is>
           <t>5th</t>
         </is>
       </c>
-      <c r="K73" s="32" t="n">
+      <c r="K75" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="L73" s="32" t="n">
+      <c r="L75" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="M73" s="32" t="n">
+      <c r="M75" s="32" t="n">
         <v>0.9330000000000001</v>
       </c>
-      <c r="N73" s="32" t="n">
+      <c r="N75" s="32" t="n">
         <v>0.8</v>
       </c>
-      <c r="O73" s="32" t="n">
+      <c r="O75" s="32" t="n">
         <v>0.7</v>
       </c>
-      <c r="P73" s="32" t="n">
+      <c r="P75" s="32" t="n">
         <v>0.781</v>
       </c>
-      <c r="Q73" s="35" t="inlineStr">
+      <c r="Q75" s="35" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>

</xml_diff>